<commit_message>
Added outputs and README
</commit_message>
<xml_diff>
--- a/Parameters/High Risk - Parameters.xlsx
+++ b/Parameters/High Risk - Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rfp437/Work/High risk/high-risk-flu/Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A137B7-281C-0C41-AF46-A8D0845C3755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112AAAC5-14AA-2348-9913-FC01A74A3800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="880" windowWidth="29040" windowHeight="15840" xr2:uid="{F6439070-539B-4A5B-A753-3646CFF84942}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{F6439070-539B-4A5B-A753-3646CFF84942}"/>
   </bookViews>
   <sheets>
     <sheet name="ConditionsList" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="MultipleConditionsSource" sheetId="3" r:id="rId4"/>
     <sheet name="MCC_Adj_Checks" sheetId="7" r:id="rId5"/>
     <sheet name="ObesitySource" sheetId="4" r:id="rId6"/>
-    <sheet name="AgeGroups" sheetId="6" r:id="rId7"/>
-    <sheet name="ChildrenObesity" sheetId="8" r:id="rId8"/>
+    <sheet name="SevereObesitySource" sheetId="9" r:id="rId7"/>
+    <sheet name="AgeGroups" sheetId="6" r:id="rId8"/>
+    <sheet name="ChildrenObesity" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="264">
   <si>
     <t>Category</t>
   </si>
@@ -797,6 +798,42 @@
   </si>
   <si>
     <t>Not in 2025 data anymore</t>
+  </si>
+  <si>
+    <t>https://www.cdc.gov/nchs/products/databriefs/db508.htm</t>
+  </si>
+  <si>
+    <t>Adults</t>
+  </si>
+  <si>
+    <t>Obese criteria</t>
+  </si>
+  <si>
+    <t>Severely obese criteria</t>
+  </si>
+  <si>
+    <t>BMI &gt;= 30</t>
+  </si>
+  <si>
+    <t>BMI &gt;= 40</t>
+  </si>
+  <si>
+    <t>SevereAmongObese</t>
+  </si>
+  <si>
+    <t>SeverelyObeseWithCondition</t>
+  </si>
+  <si>
+    <t>Proportions severely obese with some condition</t>
+  </si>
+  <si>
+    <t>Obese in US</t>
+  </si>
+  <si>
+    <t>Severely obese in US</t>
+  </si>
+  <si>
+    <t>SeverelyObeseAmongObese</t>
   </si>
 </sst>
 </file>
@@ -807,7 +844,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -832,6 +869,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -948,7 +992,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -980,6 +1024,8 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2081,18 +2127,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF81FCA5-11A4-4980-8DF6-3FB0CC39BDA0}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ObesitySource!A12</f>
         <v>0.4261084118981982</v>
+      </c>
+      <c r="B2" s="18">
+        <v>0.512459</v>
+      </c>
+      <c r="C2" s="18">
+        <v>0.23325062034739452</v>
       </c>
     </row>
   </sheetData>
@@ -3395,11 +3453,18 @@
       <c r="A11" t="s">
         <v>206</v>
       </c>
+      <c r="D11" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <f>(C6+C7)/(B6+B7)</f>
         <v>0.4261084118981982</v>
+      </c>
+      <c r="D12">
+        <f>C7/B7</f>
+        <v>0.51245886224729664</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -3462,6 +3527,72 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{777FA6C2-A4E4-7D44-B9DF-D96D0F26B020}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B2" s="17">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="D2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B3" s="17">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B4" s="17">
+        <f>B3/B2</f>
+        <v>0.23325062034739452</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B9" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>255</v>
+      </c>
+      <c r="B10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A04B9B-294C-4E9B-9670-BDEBB939213E}">
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3949,7 +4080,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8990014F-2FE6-49D1-8232-644EF7AAF89F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Replicating bar graph conditions
</commit_message>
<xml_diff>
--- a/Parameters/High Risk - Parameters.xlsx
+++ b/Parameters/High Risk - Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rfp437/Work/High risk/high-risk-flu/Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A828F4-37D6-334A-8359-CEF0B4263DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D80B44-ECA9-CC4D-8EA9-8A888E84C6C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="9" xr2:uid="{F6439070-539B-4A5B-A753-3646CFF84942}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="29040" windowHeight="15840" xr2:uid="{F6439070-539B-4A5B-A753-3646CFF84942}"/>
   </bookViews>
   <sheets>
     <sheet name="ConditionsList" sheetId="1" r:id="rId1"/>
@@ -1952,7 +1952,7 @@
         <v>79</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25">
         <v>1</v>

</xml_diff>